<commit_message>
Legal revisa la oferta y el contrato va cuando el cliente acepta
- Legal en la mesa chica ya no redacta contratos: revisa que la oferta,
  las promesas, el presupuesto y el adelanto estén dentro de la ley.
- legal_contrato.md y el flujo 6 arman el contrato a mano cuando un
  comercio acepta.
- adelanto.md: IT arma una maqueta (web, turnera, chatbot o caja) para
  los 5 mejores; queda en la pestaña Adelantos y se ve con el flujo 7.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTLhGTsTD4KZZ4pk36iN1z
</commit_message>
<xml_diff>
--- a/n8n/planilla_scaling.xlsx
+++ b/n8n/planilla_scaling.xlsx
@@ -10,15 +10,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comercios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evaluaciones" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propuestas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contratos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caja" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soporte" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adelantos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contratos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caja" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soporte" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1526,68 +1527,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>fecha</t>
+          <t>pregunta</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sesion</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>mensaje</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>respuesta</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>lead_completo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>pide_persona</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>nombre</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>comercio</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>rubro</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>zona</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>necesita</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>horario_contacto</t>
         </is>
       </c>
     </row>
@@ -1602,20 +1553,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>texto</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Scaling es una agencia de Tres de Febrero (Buenos Aires) que les arma herramientas digitales a comercios de barrio: turnos online, página web, chatbot de WhatsApp o Instagram, e inventario y caja. El dueño, Lucho, conoce cada comercio y arma un presupuesto a medida.</t>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sesion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mensaje</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>respuesta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>lead_completo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pide_persona</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>comercio</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>rubro</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>zona</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>necesita</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>horario_contacto</t>
         </is>
       </c>
     </row>
@@ -1625,6 +1624,34 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Scaling es una agencia de Tres de Febrero (Buenos Aires) que les arma herramientas digitales a comercios de barrio: turnos online, página web, chatbot de WhatsApp o Instagram, e inventario y caja. El dueño, Lucho, conoce cada comercio y arma un presupuesto a medida.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1788,7 +1815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1804,17 +1831,32 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>contrato_borrador</t>
+          <t>oferta</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>riesgos</t>
+          <t>que_va_a_ver_el_cliente</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>me_excede</t>
+          <t>legal</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>supuestos</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>html</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>revision_legal</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1840,17 +1882,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>agente</t>
+          <t>comercio</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>resumen</t>
+          <t>contrato_borrador</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>detalle</t>
+          <t>falta_completar</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>riesgos</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>me_excede</t>
         </is>
       </c>
     </row>
@@ -1865,43 +1917,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>rubro</t>
+          <t>agente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>zona</t>
+          <t>resumen</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>oferta</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>abono_mensual_ars</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>instagram</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>notas</t>
+          <t>detalle</t>
         </is>
       </c>
     </row>
@@ -1916,38 +1953,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>fecha</t>
+          <t>nombre</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>concepto</t>
+          <t>rubro</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>tipo</t>
+          <t>zona</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>monto</t>
+          <t>oferta</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>abono_mensual_ars</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>comprobante</t>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>notas</t>
         </is>
       </c>
     </row>
@@ -1962,7 +2004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1973,32 +2015,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sesion</t>
+          <t>concepto</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>mensaje</t>
+          <t>tipo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>respuesta</t>
+          <t>monto</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>resuelto</t>
+          <t>cliente</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>derivar_a_lucho</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>resumen_para_lucho</t>
+          <t>comprobante</t>
         </is>
       </c>
     </row>
@@ -2013,18 +2050,43 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>pregunta</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>sesion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mensaje</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>respuesta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>resuelto</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>derivar_a_lucho</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>resumen_para_lucho</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mesa de entrada con un Administrador de Atención y plan de implementación
- administrador_atencion.md y el flujo 8: cada 3 horas revisa las
  conversaciones terminadas de los dos chatbots, las deja en "Casos",
  pasa los interesados a Comercios y avisa por mail lo urgente.
- implementacion.md y el flujo 9: plan de trabajo de IT cuando el
  cliente firma, con las pruebas de la revisión de seguridad.
- La mesa chica saltea los comercios ya evaluados y evalúa primero los
  leads.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XTLhGTsTD4KZZ4pk36iN1z
</commit_message>
<xml_diff>
--- a/n8n/planilla_scaling.xlsx
+++ b/n8n/planilla_scaling.xlsx
@@ -12,14 +12,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propuestas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adelantos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contratos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caja" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soporte" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementaciones" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caja" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soporte" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +479,11 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>fuente</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>notas</t>
         </is>
       </c>
     </row>
@@ -511,6 +518,7 @@
           <t>https://www.openstreetmap.org/node/1178318642</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -543,6 +551,7 @@
           <t>https://www.openstreetmap.org/node/1178318657</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -575,6 +584,7 @@
           <t>https://www.openstreetmap.org/node/4394769001</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -611,6 +621,7 @@
           <t>https://www.openstreetmap.org/node/4490692290</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -643,6 +654,7 @@
           <t>https://www.openstreetmap.org/node/1178318664</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -679,6 +691,7 @@
           <t>https://www.openstreetmap.org/node/4621476642</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -711,6 +724,7 @@
           <t>https://www.openstreetmap.org/node/4621328666</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -743,6 +757,7 @@
           <t>https://www.openstreetmap.org/node/4621408945</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -775,6 +790,7 @@
           <t>https://www.openstreetmap.org/node/4626055868</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -807,6 +823,7 @@
           <t>https://www.openstreetmap.org/node/4627189527</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -839,6 +856,7 @@
           <t>https://www.openstreetmap.org/node/4627189528</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -875,6 +893,7 @@
           <t>https://www.openstreetmap.org/way/468146513</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -915,6 +934,7 @@
           <t>https://www.openstreetmap.org/node/4393505094</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -951,6 +971,7 @@
           <t>https://www.openstreetmap.org/node/4429033090</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -983,6 +1004,7 @@
           <t>https://www.openstreetmap.org/node/4626392122</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1015,6 +1037,7 @@
           <t>https://www.openstreetmap.org/node/4626982560</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1047,6 +1070,7 @@
           <t>https://www.openstreetmap.org/node/4630470631</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1079,6 +1103,7 @@
           <t>https://www.openstreetmap.org/way/468085497</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1115,6 +1140,7 @@
           <t>https://www.openstreetmap.org/node/4626529977</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1159,6 +1185,7 @@
           <t>https://www.openstreetmap.org/node/4834919621</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1191,6 +1218,7 @@
           <t>https://www.openstreetmap.org/node/4626837780</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1223,6 +1251,7 @@
           <t>https://www.openstreetmap.org/node/1239469644</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1259,6 +1288,7 @@
           <t>https://www.openstreetmap.org/node/4633465112</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1299,6 +1329,7 @@
           <t>https://www.openstreetmap.org/node/4575677216</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1335,6 +1366,7 @@
           <t>https://www.openstreetmap.org/node/4625871493</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1371,6 +1403,7 @@
           <t>https://www.openstreetmap.org/node/4625689080</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1407,6 +1440,7 @@
           <t>https://www.openstreetmap.org/node/4552646387</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1443,6 +1477,7 @@
           <t>https://www.openstreetmap.org/node/4625634101</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1479,6 +1514,7 @@
           <t>https://www.openstreetmap.org/node/4625689053</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1515,6 +1551,7 @@
           <t>https://www.openstreetmap.org/node/4625633581</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1527,18 +1564,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>pregunta</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>respuesta</t>
+          <t>concepto</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>monto</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>comprobante</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1579,42 +1636,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>lead_completo</t>
+          <t>resuelto</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>pide_persona</t>
+          <t>derivar_a_lucho</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>nombre</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>comercio</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>rubro</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>zona</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>necesita</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>horario_contacto</t>
+          <t>resumen_para_lucho</t>
         </is>
       </c>
     </row>
@@ -1629,20 +1661,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>texto</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Scaling es una agencia de Tres de Febrero (Buenos Aires) que les arma herramientas digitales a comercios de barrio: turnos online, página web, chatbot de WhatsApp o Instagram, e inventario y caja. El dueño, Lucho, conoce cada comercio y arma un presupuesto a medida.</t>
+          <t>pregunta</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>respuesta</t>
         </is>
       </c>
     </row>
@@ -1652,6 +1682,110 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sesion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mensaje</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>respuesta</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>lead_completo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>pide_persona</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>comercio</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>rubro</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>zona</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>necesita</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>horario_contacto</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Scaling es una agencia de Tres de Febrero (Buenos Aires) que les arma herramientas digitales a comercios de barrio: turnos online, página web, chatbot de WhatsApp o Instagram, e inventario y caja. El dueño, Lucho, conoce cada comercio y arma un presupuesto a medida.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1917,7 +2051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1928,15 +2062,45 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>agente</t>
+          <t>cliente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>resumen</t>
+          <t>oferta</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
+        <is>
+          <t>horas_totales</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>entrega_dia_desde_la_firma</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>tareas</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>pedir_al_comercio</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pruebas_antes_de_entregar</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>falta_antes_de_empezar</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>detalle</t>
         </is>
@@ -1953,43 +2117,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>rubro</t>
+          <t>sesion</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>zona</t>
+          <t>chatbot</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>oferta</t>
+          <t>mensajes_revisados</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>abono_mensual_ars</t>
+          <t>clasificacion</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>instagram</t>
+          <t>derivar_a</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>notas</t>
+          <t>prioridad</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>resumen</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>que_tiene_que_hacer_lucho</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>quien</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>calificacion_interesado</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>nota_chatbot</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>errores_chatbot</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>sugerencia</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>detalle</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2015,27 +2224,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>concepto</t>
+          <t>agente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>tipo</t>
+          <t>resumen</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>monto</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>cliente</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>comprobante</t>
+          <t>detalle</t>
         </is>
       </c>
     </row>
@@ -2056,37 +2255,37 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>fecha</t>
+          <t>nombre</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sesion</t>
+          <t>rubro</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>mensaje</t>
+          <t>zona</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>respuesta</t>
+          <t>oferta</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>resuelto</t>
+          <t>abono_mensual_ars</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>derivar_a_lucho</t>
+          <t>instagram</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>resumen_para_lucho</t>
+          <t>notas</t>
         </is>
       </c>
     </row>

</xml_diff>